<commit_message>
Fix day allocation formulas for low ticket counts
Co-authored-by: MaiNguyen939 <MaiNguyen939@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/estimation_28_31_may.xlsx
+++ b/estimation_28_31_may.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -619,11 +619,11 @@
         <v/>
       </c>
       <c r="D8" s="8">
-        <f>ROUND($B8*$C$5,0)</f>
+        <f>ROUND($B8*SUM($B$5:$C$5),0)-C8</f>
         <v/>
       </c>
       <c r="E8" s="8">
-        <f>ROUND($B8*$D$5,0)</f>
+        <f>ROUND($B8*SUM($B$5:$D$5),0)-C8-D8</f>
         <v/>
       </c>
       <c r="F8" s="8">
@@ -653,11 +653,11 @@
         <v/>
       </c>
       <c r="D9" s="8">
-        <f>ROUND($B9*$C$5,0)</f>
+        <f>ROUND($B9*SUM($B$5:$C$5),0)-C9</f>
         <v/>
       </c>
       <c r="E9" s="8">
-        <f>ROUND($B9*$D$5,0)</f>
+        <f>ROUND($B9*SUM($B$5:$D$5),0)-C9-D9</f>
         <v/>
       </c>
       <c r="F9" s="8">
@@ -687,11 +687,11 @@
         <v/>
       </c>
       <c r="D10" s="8">
-        <f>ROUND($B10*$C$5,0)</f>
+        <f>ROUND($B10*SUM($B$5:$C$5),0)-C10</f>
         <v/>
       </c>
       <c r="E10" s="8">
-        <f>ROUND($B10*$D$5,0)</f>
+        <f>ROUND($B10*SUM($B$5:$D$5),0)-C10-D10</f>
         <v/>
       </c>
       <c r="F10" s="8">
@@ -721,11 +721,11 @@
         <v/>
       </c>
       <c r="D11" s="8">
-        <f>ROUND($B11*$C$5,0)</f>
+        <f>ROUND($B11*SUM($B$5:$C$5),0)-C11</f>
         <v/>
       </c>
       <c r="E11" s="8">
-        <f>ROUND($B11*$D$5,0)</f>
+        <f>ROUND($B11*SUM($B$5:$D$5),0)-C11-D11</f>
         <v/>
       </c>
       <c r="F11" s="8">
@@ -755,11 +755,11 @@
         <v/>
       </c>
       <c r="D12" s="8">
-        <f>ROUND($B12*$C$5,0)</f>
+        <f>ROUND($B12*SUM($B$5:$C$5),0)-C12</f>
         <v/>
       </c>
       <c r="E12" s="8">
-        <f>ROUND($B12*$D$5,0)</f>
+        <f>ROUND($B12*SUM($B$5:$D$5),0)-C12-D12</f>
         <v/>
       </c>
       <c r="F12" s="8">
@@ -828,6 +828,13 @@
       <c r="A16" t="inlineStr">
         <is>
           <t>- Neu F5 khac 100%, phan bo chua can bang.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>- Cong thuc lam tron luy ke tranh am ticket o ngay cuoi.</t>
         </is>
       </c>
     </row>

</xml_diff>